<commit_message>
Doku und kleine Änderungen
</commit_message>
<xml_diff>
--- a/Testdaten.xlsx
+++ b/Testdaten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jan-s\PycharmProjects\Adressliste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E9EF63-C9F7-4E70-A641-7A6BB12EDE81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1790D02-C471-429A-B708-A28DD0FD8C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DFFF17E1-0C00-426B-9CA3-ACCBC61A4D01}"/>
+    <workbookView xWindow="-22230" yWindow="2025" windowWidth="17280" windowHeight="8880" xr2:uid="{DFFF17E1-0C00-426B-9CA3-ACCBC61A4D01}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
-    <t>Das ist eine Testseite</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t>Ort</t>
   </si>
   <si>
-    <t>Amt</t>
-  </si>
-  <si>
     <t>E-Mail privat</t>
   </si>
   <si>
@@ -65,9 +59,6 @@
     <t>Telefon</t>
   </si>
   <si>
-    <t>Handlanger</t>
-  </si>
-  <si>
     <t>Max</t>
   </si>
   <si>
@@ -77,15 +68,6 @@
     <t>Musterhausen</t>
   </si>
   <si>
-    <t>abc@def.gh</t>
-  </si>
-  <si>
-    <t>123@asdf.ghj</t>
-  </si>
-  <si>
-    <t>086423-5643</t>
-  </si>
-  <si>
     <t>Str.</t>
   </si>
   <si>
@@ -98,43 +80,61 @@
     <t>Hauptstr.</t>
   </si>
   <si>
-    <t>Dortmund</t>
-  </si>
-  <si>
-    <t>Doris</t>
-  </si>
-  <si>
-    <t>Bochum</t>
-  </si>
-  <si>
-    <t>Tante</t>
-  </si>
-  <si>
-    <t>dd@bochuum.com</t>
-  </si>
-  <si>
     <t>0160/123456789</t>
   </si>
   <si>
-    <t>Fischer</t>
-  </si>
-  <si>
-    <t>Fritz</t>
-  </si>
-  <si>
-    <t>Frankfurt</t>
-  </si>
-  <si>
-    <t>Fasanenzüchter</t>
-  </si>
-  <si>
-    <t>0987654@poiuztr.ew</t>
-  </si>
-  <si>
     <t>Kleiner Weg</t>
   </si>
   <si>
     <t>Geburtsdatum</t>
+  </si>
+  <si>
+    <t>Beruf</t>
+  </si>
+  <si>
+    <t>Maurer</t>
+  </si>
+  <si>
+    <t>MM@example.com</t>
+  </si>
+  <si>
+    <t>Max@example.com</t>
+  </si>
+  <si>
+    <t>011223-45678</t>
+  </si>
+  <si>
+    <t>Albrecht</t>
+  </si>
+  <si>
+    <t>Anton</t>
+  </si>
+  <si>
+    <t>Aachen</t>
+  </si>
+  <si>
+    <t>Arzt</t>
+  </si>
+  <si>
+    <t>aa@example.com</t>
+  </si>
+  <si>
+    <t>Brecht</t>
+  </si>
+  <si>
+    <t>Berta</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Beamtin</t>
+  </si>
+  <si>
+    <t>BB@example.com</t>
+  </si>
+  <si>
+    <t>Das ist eine Testtabelle.</t>
   </si>
 </sst>
 </file>
@@ -555,15 +555,16 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -576,66 +577,66 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="I3" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E4" s="4">
         <v>18614</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="J4" s="2">
         <v>17</v>
@@ -646,24 +647,24 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -671,27 +672,27 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="4">
         <v>40391</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="J6" s="2">
         <v>3</v>

</xml_diff>